<commit_message>
Publish 167-centre-ave-r4 (demo, link only): 167-centre-ave-seller-net-proceeds.xlsx
</commit_message>
<xml_diff>
--- a/p/167-centre-ave-0a01cc/167-centre-ave-seller-net-proceeds.xlsx
+++ b/p/167-centre-ave-0a01cc/167-centre-ave-seller-net-proceeds.xlsx
@@ -565,7 +565,7 @@
         <v>600000</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>665000</v>
+        <v>675000</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -582,7 +582,7 @@
       </c>
       <c r="D9" s="6" t="n">
         <f aca="false">ROUND(IF(ROUND(D8,2)&lt;=350000,IF($B$6="YES",ROUNDUP(MAX(0,MIN(ROUND(D8,2),150000)-0)/500,0)*0.5+ROUNDUP(MAX(0,MIN(ROUND(D8,2),350000)-150000)/500,0)*1.25,ROUNDUP(MAX(0,MIN(ROUND(D8,2),150000)-0)/500,0)*2+ROUNDUP(MAX(0,MIN(ROUND(D8,2),200000)-150000)/500,0)*3.35+ROUNDUP(MAX(0,MIN(ROUND(D8,2),350000)-200000)/500,0)*3.9),IF($B$6="YES",ROUNDUP(MAX(0,MIN(ROUND(D8,2),150000)-0)/500,0)*1.4+ROUNDUP(MAX(0,MIN(ROUND(D8,2),550000)-150000)/500,0)*2.15+ROUNDUP(MAX(0,MIN(ROUND(D8,2),850000)-550000)/500,0)*2.65+ROUNDUP(MAX(0,MIN(ROUND(D8,2),1000000)-850000)/500,0)*3.15+ROUNDUP(MAX(0,ROUND(D8,2)-1000000)/500,0)*3.4,ROUNDUP(MAX(0,MIN(ROUND(D8,2),150000)-0)/500,0)*2.9+ROUNDUP(MAX(0,MIN(ROUND(D8,2),200000)-150000)/500,0)*4.25+ROUNDUP(MAX(0,MIN(ROUND(D8,2),550000)-200000)/500,0)*4.8+ROUNDUP(MAX(0,MIN(ROUND(D8,2),850000)-550000)/500,0)*5.3+ROUNDUP(MAX(0,MIN(ROUND(D8,2),1000000)-850000)/500,0)*5.8+ROUNDUP(MAX(0,ROUND(D8,2)-1000000)/500,0)*6.05)),2)</f>
-        <v>5874</v>
+        <v>5980</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -616,7 +616,7 @@
       </c>
       <c r="D11" s="6" t="n">
         <f aca="false">ROUND($B$5*ROUND(D8,2),2)</f>
-        <v>26600</v>
+        <v>27000</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -675,7 +675,7 @@
       </c>
       <c r="D15" s="6" t="n">
         <f aca="false">ROUND(ROUND(D8,2)-SUM(D9:D11)-ROUND(D12,2)-ROUND(D13,2)-ROUND(D14,2),2)</f>
-        <v>630826</v>
+        <v>640320</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -706,7 +706,7 @@
       </c>
       <c r="D17" s="6" t="n">
         <f aca="false">ROUND(D15-IF(ISNUMBER(D16),ROUND(D16,2),0),2)</f>
-        <v>630826</v>
+        <v>640320</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>